<commit_message>
resolved error message failure
</commit_message>
<xml_diff>
--- a/testData/testdata.xlsx
+++ b/testData/testdata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Amruta\PlaywrightTest\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01091285-1868-48AA-96D7-224DCD9D5E95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC298247-B9EA-4A7B-BDCD-E6137A588A89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Checkout" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="19">
   <si>
     <t>testName</t>
   </si>
@@ -68,6 +68,21 @@
   </si>
   <si>
     <t>Missing First Name</t>
+  </si>
+  <si>
+    <t>Error: Last Name is required</t>
+  </si>
+  <si>
+    <t>Error: Postal Code is required</t>
+  </si>
+  <si>
+    <t>Error: First Name is required</t>
+  </si>
+  <si>
+    <t>Missing Last Name</t>
+  </si>
+  <si>
+    <t>errormessage</t>
   </si>
 </sst>
 </file>
@@ -465,14 +480,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFE22F8B-C3C4-4B5F-99E9-A23A8F8F6091}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23.81640625" customWidth="1"/>
     <col min="3" max="3" width="13.1796875" customWidth="1"/>
+    <col min="6" max="6" width="27.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -488,10 +504,13 @@
       <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F1" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>11</v>
@@ -499,24 +518,46 @@
       <c r="C2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" s="2"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D2" s="2"/>
+      <c r="E2" s="2">
+        <v>400001</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="2"/>
+      <c r="C3" s="2" t="s">
+        <v>8</v>
+      </c>
       <c r="D3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="2">
-        <v>400001</v>
+      <c r="F3" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4">
+        <v>34345</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>